<commit_message>
Added complete baseline and desc stats
</commit_message>
<xml_diff>
--- a/results/intensive_baseline_weighted/original/log_intensive_baseline_weighted_b1_1000perm.xlsx
+++ b/results/intensive_baseline_weighted/original/log_intensive_baseline_weighted_b1_1000perm.xlsx
@@ -351,59 +351,147 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>total_shares</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>total_comments</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>total_reactions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>ver</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>non_ver</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fake</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>n_posts</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>eng</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>n_posts_covid</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>pos_b_covid</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>neutral_b_covid</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>neg_b_covid</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>n_posts_vax</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>pos_b_vax</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>neutral_b_vax</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>neg_b_vax</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2">
+        <v>-0.07754878899015853</v>
+      </c>
+      <c r="B2">
+        <v>-0.04661670830767476</v>
+      </c>
+      <c r="C2">
+        <v>-0.06578978290827373</v>
+      </c>
+      <c r="D2">
         <v>-0.02432896839972535</v>
       </c>
-      <c r="B2">
+      <c r="E2">
         <v>-0.02723338439036652</v>
       </c>
-      <c r="C2">
+      <c r="F2">
         <v>-0.02986210513112132</v>
       </c>
-      <c r="D2">
+      <c r="G2">
         <v>-0.005881103233681505</v>
       </c>
-      <c r="E2">
+      <c r="H2">
         <v>-0.006595473409398987</v>
       </c>
-      <c r="F2">
+      <c r="I2">
         <v>-0.03236837128187898</v>
+      </c>
+      <c r="J2">
+        <v>0.0002029681830579248</v>
+      </c>
+      <c r="K2">
+        <v>-0.0006331694805541167</v>
+      </c>
+      <c r="L2">
+        <v>-0.0008181414378754658</v>
+      </c>
+      <c r="M2">
+        <v>0.003049423634707434</v>
+      </c>
+      <c r="N2">
+        <v>-0.0001923922146082593</v>
+      </c>
+      <c r="O2">
+        <v>-0.0002443002063760789</v>
+      </c>
+      <c r="P2">
+        <v>5.489158270883098e-05</v>
+      </c>
+      <c r="Q2">
+        <v>0.0006114952105265598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>